<commit_message>
Added ECO slides and ECO outline
</commit_message>
<xml_diff>
--- a/PMP_30_Day_Study_Plan.xlsx
+++ b/PMP_30_Day_Study_Plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eric.hayes\Documents\PMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CB565403-1C1C-403A-8685-DCFD88E1B14F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{496A9489-92D4-4D1E-90C0-3E3652F293C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-12630" yWindow="-16320" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="30-Day Study Plan" sheetId="1" r:id="rId1"/>
@@ -485,7 +485,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -517,6 +517,14 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+      <extLst>
+        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement i="0"/>
+        </ext>
+      </extLst>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -532,6 +540,23 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<FeaturePropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <bag type="Checkbox"/>
+  <bag type="XFControls">
+    <bagId k="CellControl">0</bagId>
+  </bag>
+  <bag type="XFComplement">
+    <bagId k="XFControls">1</bagId>
+  </bag>
+  <bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <a k="MappedFeaturePropertyBags">
+      <bagId>2</bagId>
+    </a>
+  </bag>
+</FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -875,7 +900,9 @@
         <v>11</v>
       </c>
       <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="G2" s="13" t="b">
+        <v>1</v>
+      </c>
       <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -895,7 +922,9 @@
         <v>13</v>
       </c>
       <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
+      <c r="G3" s="13" t="b">
+        <v>1</v>
+      </c>
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -915,7 +944,9 @@
         <v>16</v>
       </c>
       <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
+      <c r="G4" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -935,7 +966,9 @@
         <v>18</v>
       </c>
       <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
+      <c r="G5" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -957,7 +990,9 @@
       <c r="F6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="2"/>
+      <c r="G6" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -977,7 +1012,9 @@
         <v>25</v>
       </c>
       <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
+      <c r="G7" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -997,7 +1034,9 @@
         <v>28</v>
       </c>
       <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+      <c r="G8" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1017,7 +1056,9 @@
         <v>32</v>
       </c>
       <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
+      <c r="G9" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1037,7 +1078,9 @@
         <v>34</v>
       </c>
       <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+      <c r="G10" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H10" s="4"/>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1059,7 +1102,9 @@
       <c r="F11" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G11" s="2"/>
+      <c r="G11" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H11" s="4"/>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1079,7 +1124,9 @@
         <v>40</v>
       </c>
       <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+      <c r="G12" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H12" s="4"/>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1099,7 +1146,9 @@
         <v>43</v>
       </c>
       <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+      <c r="G13" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H13" s="4"/>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1119,7 +1168,9 @@
         <v>45</v>
       </c>
       <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+      <c r="G14" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H14" s="4"/>
     </row>
     <row r="15" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1139,7 +1190,9 @@
         <v>48</v>
       </c>
       <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+      <c r="G15" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H15" s="4"/>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1161,7 +1214,9 @@
       <c r="F16" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G16" s="2"/>
+      <c r="G16" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H16" s="4"/>
     </row>
     <row r="17" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1181,7 +1236,9 @@
         <v>54</v>
       </c>
       <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
+      <c r="G17" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H17" s="4"/>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1201,7 +1258,9 @@
         <v>57</v>
       </c>
       <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="G18" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H18" s="4"/>
     </row>
     <row r="19" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1221,7 +1280,9 @@
         <v>59</v>
       </c>
       <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
+      <c r="G19" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H19" s="4"/>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1243,7 +1304,9 @@
       <c r="F20" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="G20" s="2"/>
+      <c r="G20" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H20" s="4"/>
     </row>
     <row r="21" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1263,7 +1326,9 @@
         <v>63</v>
       </c>
       <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+      <c r="G21" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H21" s="4"/>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1283,7 +1348,9 @@
         <v>66</v>
       </c>
       <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
+      <c r="G22" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H22" s="4"/>
     </row>
     <row r="23" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1305,7 +1372,9 @@
       <c r="F23" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G23" s="2"/>
+      <c r="G23" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H23" s="4"/>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1325,7 +1394,9 @@
         <v>72</v>
       </c>
       <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
+      <c r="G24" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H24" s="4"/>
     </row>
     <row r="25" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1347,7 +1418,9 @@
       <c r="F25" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="G25" s="2"/>
+      <c r="G25" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H25" s="4"/>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1367,7 +1440,9 @@
         <v>76</v>
       </c>
       <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
+      <c r="G26" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H26" s="4"/>
     </row>
     <row r="27" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1387,7 +1462,9 @@
         <v>79</v>
       </c>
       <c r="F27" s="2"/>
-      <c r="G27" s="2"/>
+      <c r="G27" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H27" s="4"/>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1407,7 +1484,9 @@
         <v>81</v>
       </c>
       <c r="F28" s="2"/>
-      <c r="G28" s="2"/>
+      <c r="G28" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H28" s="4"/>
     </row>
     <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1429,7 +1508,9 @@
       <c r="F29" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="G29" s="2"/>
+      <c r="G29" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H29" s="4"/>
     </row>
     <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1449,7 +1530,9 @@
         <v>88</v>
       </c>
       <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
+      <c r="G30" s="13" t="b">
+        <v>0</v>
+      </c>
       <c r="H30" s="4"/>
     </row>
     <row r="31" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>